<commit_message>
update: replace Hem catalogue with latest version (Hem catalogue 3)
</commit_message>
<xml_diff>
--- a/Hem catalogue.xlsx
+++ b/Hem catalogue.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maa00\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C40AC16-E664-43D3-B4E5-5635B7273333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC72B4D2-BDDD-4DF5-9F81-C29513F9C8AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hem catalogue'!$A$1:$G$722</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5363" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5363" uniqueCount="934">
   <si>
     <t>Category</t>
   </si>
@@ -2826,22 +2826,28 @@
     <t>SMC - Smudge Tin  Candle White Sage</t>
   </si>
   <si>
-    <t>Black Current Car Freshner</t>
-  </si>
-  <si>
-    <t>Citrus Breeze Car Freshner</t>
-  </si>
-  <si>
-    <t>Dreamy Rose Car Freshner</t>
-  </si>
-  <si>
-    <t>Fresh Bergamote Car Freshner</t>
-  </si>
-  <si>
-    <t>Peach Blossom Car Freshner</t>
-  </si>
-  <si>
-    <t>Aqua Car Freshner</t>
+    <t>CAR FRESHENER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Cherry Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Current Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citrus Breeze Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dreamy Rose Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh Bergamote Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aqua Car Freshener </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peach Blossom Car Freshener </t>
   </si>
 </sst>
 </file>
@@ -5061,11 +5067,11 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="3" t="s">
-        <v>768</v>
+        <v>927</v>
       </c>
       <c r="D56" s="16" t="s">
         <v>821</v>
@@ -5074,22 +5080,22 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="3" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="D57" s="16"/>
       <c r="E57" s="2"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="3" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="D58" s="16" t="s">
         <v>822</v>
@@ -5098,11 +5104,11 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="3" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="D59" s="16" t="s">
         <v>823</v>
@@ -5111,33 +5117,33 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="3" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="D60" s="16"/>
       <c r="E60" s="2"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="3" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="D61" s="16"/>
       <c r="E61" s="2"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>766</v>
+        <v>926</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="3" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
       <c r="D62" s="16" t="s">
         <v>824</v>

</xml_diff>